<commit_message>
Nana match 19 (3-0) in spreadsheet
</commit_message>
<xml_diff>
--- a/FamilyWorldCup2026.xlsx
+++ b/FamilyWorldCup2026.xlsx
@@ -3090,8 +3090,12 @@
         <f>IF(OR(I22="",J22="",$G22="",$H22=""),0,IF(AND(I22=$G22,J22=$H22),8,IF(SIGN(I22-J22)=SIGN($G22-$H22),3,0)))</f>
         <v/>
       </c>
-      <c r="L22" s="66" t="n"/>
-      <c r="M22" s="66" t="n"/>
+      <c r="L22" s="66" t="n">
+        <v>3</v>
+      </c>
+      <c r="M22" s="66" t="n">
+        <v>0</v>
+      </c>
       <c r="N22" s="67">
         <f>IF(OR(L22="",M22="",$G22="",$H22=""),0,IF(AND(L22=$G22,M22=$H22),8,IF(SIGN(L22-M22)=SIGN($G22-$H22),3,0)))</f>
         <v/>

</xml_diff>